<commit_message>
05/06: clarify readme/starter instructions so they match the workbook scaffolding (pre-filled vs response cells, exception flow, escalation spec, workflow output columns). one over-specific count dropped from a solution markdown cell.
</commit_message>
<xml_diff>
--- a/06_ai-incident-response-playbook-simulation/exercises/starter/incident_response_starter.xlsx
+++ b/06_ai-incident-response-playbook-simulation/exercises/starter/incident_response_starter.xlsx
@@ -2148,15 +2148,20 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
+          <t>Postmortem Report Template</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Zoom, Confluence, Jira</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>"Postmortem document with timeline, root cause, contributing factors, action items with owners and deadlines"
 Reasoning: Structured documentation ensures completeness; clear ownership and deadlines drive accountability; shared document enables transparency and organizational learning.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Zoom, Confluence, Jira</t>
-        </is>
-      </c>
       <c r="H10" s="19" t="inlineStr">
         <is>
           <t>[Your response here — for Step 9 Post-Incident Review: do you actually run blameless postmortems in Confluence or Jira, is the 48-hour window enforced, and does Product or Data Science Lead actually attend or send a delegate?]</t>
@@ -2189,13 +2194,18 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
+          <t>Runbook / KB Update Template</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Confluence, GitHub Wiki</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>"Updated runbooks in Confluence, new alerting rules in monitoring system, root cause article in knowledge base"
 Reasoning: Confluence ensures team can find procedures; updated alerts prevent recurrence; knowledge base article enables transfer of learning across organization.</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Confluence, GitHub Wiki</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">

</xml_diff>